<commit_message>
updated supplier import columns
</commit_message>
<xml_diff>
--- a/fmt/tests/suppliers_import.xlsx
+++ b/fmt/tests/suppliers_import.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEV\wamp64\www\fmt-yb\packages\fmt\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57CCEC5C-3A1D-42C5-B74B-392DB05E05C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D107A531-EA29-49E8-A4C4-0308E9957246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="45" windowWidth="28800" windowHeight="15435" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="62">
   <si>
     <t>legal_name</t>
   </si>
@@ -51,27 +51,15 @@
     <t>phone_2</t>
   </si>
   <si>
-    <t>phone_3</t>
-  </si>
-  <si>
     <t>email_1</t>
   </si>
   <si>
     <t>email_2</t>
   </si>
   <si>
-    <t>email_3</t>
-  </si>
-  <si>
-    <t>Bic_1</t>
-  </si>
-  <si>
     <t>iban_1</t>
   </si>
   <si>
-    <t>bic_2</t>
-  </si>
-  <si>
     <t>iban_2</t>
   </si>
   <si>
@@ -102,9 +90,6 @@
     <t>supplier1@mail.com</t>
   </si>
   <si>
-    <t>BBRUBEBB</t>
-  </si>
-  <si>
     <t>BE42589710346621</t>
   </si>
   <si>
@@ -156,9 +141,6 @@
     <t>024568972</t>
   </si>
   <si>
-    <t>GKCCBEBB</t>
-  </si>
-  <si>
     <t>BE91742055681934</t>
   </si>
   <si>
@@ -216,9 +198,6 @@
     <t>supplier5accounting@mail.com</t>
   </si>
   <si>
-    <t>supplier5finance@mail.com</t>
-  </si>
-  <si>
     <t>BE28684399104578</t>
   </si>
   <si>
@@ -226,6 +205,12 @@
   </si>
   <si>
     <t>0826091475</t>
+  </si>
+  <si>
+    <t>mobile_1</t>
+  </si>
+  <si>
+    <t>iban_3</t>
   </si>
 </sst>
 </file>
@@ -388,10 +373,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -417,227 +402,203 @@
         <v>7</v>
       </c>
       <c r="I1" t="s">
+        <v>60</v>
+      </c>
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
+        <v>61</v>
+      </c>
+      <c r="O1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="P1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="B2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="C2" t="s">
         <v>16</v>
-      </c>
-      <c r="R1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" t="s">
-        <v>20</v>
       </c>
       <c r="D2">
         <v>1120</v>
       </c>
       <c r="E2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" t="s">
         <v>21</v>
       </c>
-      <c r="F2" t="s">
+      <c r="O2" t="s">
         <v>22</v>
       </c>
-      <c r="G2" t="s">
+      <c r="P2" t="s">
         <v>23</v>
       </c>
-      <c r="J2" t="s">
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>24</v>
       </c>
-      <c r="M2" t="s">
+      <c r="B3" t="s">
         <v>25</v>
       </c>
-      <c r="N2" t="s">
+      <c r="C3" t="s">
         <v>26</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>27</v>
-      </c>
-      <c r="R2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" t="s">
-        <v>31</v>
       </c>
       <c r="D3">
         <v>1160</v>
       </c>
       <c r="E3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" t="s">
+        <v>29</v>
+      </c>
+      <c r="L3" t="s">
+        <v>30</v>
+      </c>
+      <c r="O3" t="s">
+        <v>31</v>
+      </c>
+      <c r="P3" t="s">
         <v>32</v>
       </c>
-      <c r="F3" t="s">
-        <v>22</v>
-      </c>
-      <c r="G3" t="s">
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>33</v>
       </c>
-      <c r="J3" t="s">
+      <c r="B4" t="s">
         <v>34</v>
       </c>
-      <c r="M3" t="s">
-        <v>25</v>
-      </c>
-      <c r="N3" t="s">
+      <c r="C4" t="s">
         <v>35</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>36</v>
-      </c>
-      <c r="R3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C4" t="s">
-        <v>40</v>
       </c>
       <c r="D4">
         <v>1020</v>
       </c>
       <c r="E4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" t="s">
+        <v>37</v>
+      </c>
+      <c r="L4" t="s">
+        <v>38</v>
+      </c>
+      <c r="O4" t="s">
+        <v>39</v>
+      </c>
+      <c r="P4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>41</v>
       </c>
-      <c r="F4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="B5" t="s">
         <v>42</v>
       </c>
-      <c r="M4" t="s">
+      <c r="C5" t="s">
         <v>43</v>
-      </c>
-      <c r="N4" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>45</v>
-      </c>
-      <c r="R4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>47</v>
-      </c>
-      <c r="B5" t="s">
-        <v>48</v>
-      </c>
-      <c r="C5" t="s">
-        <v>49</v>
       </c>
       <c r="D5">
         <v>1315</v>
       </c>
       <c r="E5" t="s">
+        <v>44</v>
+      </c>
+      <c r="F5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" t="s">
+        <v>45</v>
+      </c>
+      <c r="J5" t="s">
+        <v>46</v>
+      </c>
+      <c r="L5" t="s">
+        <v>47</v>
+      </c>
+      <c r="O5" t="s">
+        <v>48</v>
+      </c>
+      <c r="P5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>50</v>
       </c>
-      <c r="F5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="B6" t="s">
         <v>51</v>
       </c>
-      <c r="J5" t="s">
+      <c r="C6" t="s">
         <v>52</v>
-      </c>
-      <c r="M5" t="s">
-        <v>25</v>
-      </c>
-      <c r="N5" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>54</v>
-      </c>
-      <c r="R5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B6" t="s">
-        <v>57</v>
-      </c>
-      <c r="C6" t="s">
-        <v>58</v>
       </c>
       <c r="D6">
         <v>1000</v>
       </c>
       <c r="E6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" t="s">
+        <v>54</v>
+      </c>
+      <c r="J6" t="s">
+        <v>55</v>
+      </c>
+      <c r="K6" t="s">
+        <v>56</v>
+      </c>
+      <c r="L6" t="s">
+        <v>57</v>
+      </c>
+      <c r="O6" t="s">
+        <v>58</v>
+      </c>
+      <c r="P6" t="s">
         <v>59</v>
-      </c>
-      <c r="F6" t="s">
-        <v>22</v>
-      </c>
-      <c r="G6" t="s">
-        <v>60</v>
-      </c>
-      <c r="J6" t="s">
-        <v>61</v>
-      </c>
-      <c r="K6" t="s">
-        <v>62</v>
-      </c>
-      <c r="L6" t="s">
-        <v>63</v>
-      </c>
-      <c r="M6" t="s">
-        <v>43</v>
-      </c>
-      <c r="N6" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>65</v>
-      </c>
-      <c r="R6" t="s">
-        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>